<commit_message>
Model PG adjacency and sync verified submission package
</commit_message>
<xml_diff>
--- a/Campus_Store_Model.xlsx
+++ b/Campus_Store_Model.xlsx
@@ -559,10 +559,10 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>352</v>
+        <v>366</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>352</v>
+        <v>366</v>
       </c>
       <c r="D6" s="5">
         <f>IF(B6=C6,"PASS","FAIL")</f>
@@ -640,10 +640,10 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>167</v>
+        <v>183</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>167</v>
+        <v>183</v>
       </c>
       <c r="D9" s="5">
         <f>IF(B9=C9,"PASS","FAIL")</f>
@@ -667,10 +667,10 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D10" s="5">
         <f>IF(B10=C10,"PASS","FAIL")</f>

</xml_diff>

<commit_message>
Add evidence-gated PG adjacency scenario
</commit_message>
<xml_diff>
--- a/Campus_Store_Model.xlsx
+++ b/Campus_Store_Model.xlsx
@@ -16,6 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 Risks" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7 District Screen" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8 Verification" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9 PG Adjacency" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +25,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+  </numFmts>
   <fonts count="6">
     <font>
       <name val="Calibri"/>
@@ -63,7 +67,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -83,6 +87,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDCE7F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC220"/>
       </patternFill>
     </fill>
     <fill>
@@ -108,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -121,8 +130,15 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -559,10 +575,10 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>366</v>
+        <v>378</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>366</v>
+        <v>378</v>
       </c>
       <c r="D6" s="5">
         <f>IF(B6=C6,"PASS","FAIL")</f>
@@ -640,10 +656,10 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D9" s="5">
         <f>IF(B9=C9,"PASS","FAIL")</f>
@@ -667,10 +683,10 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="D10" s="5">
         <f>IF(B10=C10,"PASS","FAIL")</f>
@@ -692,6 +708,862 @@
         <is>
           <t>ALL FIVE LAYERS PASSED on the last recorded run.</t>
         </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:H2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PG adjacency — evidence-gated demand and capacity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>The hostel-only base case is unchanged. PG demand enters only after the evidence gate opens, and only into spare term capacity or available break-period capacity. Edit the gold pilot inputs on 1 Inputs; every output below is a live formula.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>CONFIGURED SCENARIO — ZERO UNTIL THE PILOT INPUTS ARE EVIDENCED</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Decision reading</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>PG demand evidence status</t>
+        </is>
+      </c>
+      <c r="B6" s="11">
+        <f>IF(AND('1 Inputs'!$B$19=TRUE,'1 Inputs'!$B$20&gt;0,'1 Inputs'!$B$21&gt;0,'1 Inputs'!$B$22&gt;0),"OPEN","CLOSED")</f>
+        <v/>
+      </c>
+      <c r="C6" s="11" t="inlineStr"/>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>CLOSED means PG contributes zero to every published return</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Gross PG demand</t>
+        </is>
+      </c>
+      <c r="B7" s="12">
+        <f>IF(AND('1 Inputs'!$B$19=TRUE,'1 Inputs'!$B$20&gt;0,'1 Inputs'!$B$21&gt;0,'1 Inputs'!$B$22&gt;0),'1 Inputs'!$B$20*'1 Inputs'!$B$21*'1 Inputs'!$B$26,0)</f>
+        <v/>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>orders/day</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>verified beds × active-user penetration × frequency</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Spare term capacity</t>
+        </is>
+      </c>
+      <c r="B8" s="12">
+        <f>MAX(0,'1 Inputs'!$B$5-'1 Inputs'!$B$25)</f>
+        <v/>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>orders/day</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>PG is not added above the store working ceiling</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>PG admitted in term</t>
+        </is>
+      </c>
+      <c r="B9" s="12">
+        <f>MIN(B7,B8)</f>
+        <v/>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>orders/day</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>the lower of evidenced demand and spare capacity</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>PG overflow / capacity trigger</t>
+        </is>
+      </c>
+      <c r="B10" s="12">
+        <f>MAX(0,B7-B9)</f>
+        <v/>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>orders/day</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>requires capacity expansion or remains unserved</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>PG admitted in academic break</t>
+        </is>
+      </c>
+      <c r="B11" s="12">
+        <f>MIN('1 Inputs'!$B$5,B7*'1 Inputs'!$B$24)</f>
+        <v/>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>orders/day</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>zero until break retention is measured</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Weighted PG last mile</t>
+        </is>
+      </c>
+      <c r="B12" s="13">
+        <f>(1-'1 Inputs'!$B$23)*'1 Inputs'!$B$27+'1 Inputs'!$B$23*'1 Inputs'!$B$28</f>
+        <v/>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Rs/order</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>doorstep/common-drop mix</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>PG contribution per order</t>
+        </is>
+      </c>
+      <c r="B13" s="13">
+        <f>IF('1 Inputs'!$B$22&gt;0,'1 Inputs'!$B$8*'1 Inputs'!$B$22-B12-'1 Inputs'!$B$10-'1 Inputs'!$B$11-'1 Inputs'!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Rs/order</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>same take rate and store-cost basis as the core model</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Annual incremental PG orders</t>
+        </is>
+      </c>
+      <c r="B14" s="14">
+        <f>B9*'1 Inputs'!$B$30+B11*'1 Inputs'!$B$31</f>
+        <v/>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>orders/year</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>term spare capacity plus measured break retention</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Incremental PG EBIT</t>
+        </is>
+      </c>
+      <c r="B15" s="14">
+        <f>B14*B13</f>
+        <v/>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Rs/year</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>before any capacity-expansion capex</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Incremental PG working capital</t>
+        </is>
+      </c>
+      <c r="B16" s="14">
+        <f>MAX(B9,B11)*'1 Inputs'!$B$22*'1 Inputs'!$B$29*'1 Inputs'!$B$15</f>
+        <v/>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Rs</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>14 NWC days on incremental NOV</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Base EBIT at configured hostel volume</t>
+        </is>
+      </c>
+      <c r="B17" s="14">
+        <f>('1 Inputs'!$B$8*'1 Inputs'!$B$32-'1 Inputs'!$B$13-'1 Inputs'!$B$14-'1 Inputs'!$B$10-'1 Inputs'!$B$11-'1 Inputs'!$B$12)*'1 Inputs'!$B$25*'1 Inputs'!$B$30-'1 Inputs'!$B$9*12</f>
+        <v/>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Rs/year</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>30% non-grocery AOV comparison basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Pro-forma node ROCE</t>
+        </is>
+      </c>
+      <c r="B18" s="15">
+        <f>(B17+B15)/('1 Inputs'!$B$16+'1 Inputs'!$B$15*'1 Inputs'!$B$5*'1 Inputs'!$B$32*'1 Inputs'!$B$29+B16)</f>
+        <v/>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>PG changes the return only after the evidence gate opens</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>NORMALISED CAPACITY SENSITIVITY — PER 1,000 VERIFIED OCCUPIED STUDENT BEDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Active-user penetration</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Hostel orders/day</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Gross PG orders/day</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Spare capacity</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>PG served</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>PG overflow</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B23" s="12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C23" s="12">
+        <f>1000*A23*'1 Inputs'!$B$26</f>
+        <v/>
+      </c>
+      <c r="D23" s="12">
+        <f>MAX(0,'1 Inputs'!$B$5-B23)</f>
+        <v/>
+      </c>
+      <c r="E23" s="12">
+        <f>MIN(C23,D23)</f>
+        <v/>
+      </c>
+      <c r="F23" s="12">
+        <f>MAX(0,C23-E23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B24" s="12" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C24" s="12">
+        <f>1000*A24*'1 Inputs'!$B$26</f>
+        <v/>
+      </c>
+      <c r="D24" s="12">
+        <f>MAX(0,'1 Inputs'!$B$5-B24)</f>
+        <v/>
+      </c>
+      <c r="E24" s="12">
+        <f>MIN(C24,D24)</f>
+        <v/>
+      </c>
+      <c r="F24" s="12">
+        <f>MAX(0,C24-E24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B25" s="12" t="n">
+        <v>1400</v>
+      </c>
+      <c r="C25" s="12">
+        <f>1000*A25*'1 Inputs'!$B$26</f>
+        <v/>
+      </c>
+      <c r="D25" s="12">
+        <f>MAX(0,'1 Inputs'!$B$5-B25)</f>
+        <v/>
+      </c>
+      <c r="E25" s="12">
+        <f>MIN(C25,D25)</f>
+        <v/>
+      </c>
+      <c r="F25" s="12">
+        <f>MAX(0,C25-E25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="16" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="B26" s="12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C26" s="12">
+        <f>1000*A26*'1 Inputs'!$B$26</f>
+        <v/>
+      </c>
+      <c r="D26" s="12">
+        <f>MAX(0,'1 Inputs'!$B$5-B26)</f>
+        <v/>
+      </c>
+      <c r="E26" s="12">
+        <f>MIN(C26,D26)</f>
+        <v/>
+      </c>
+      <c r="F26" s="12">
+        <f>MAX(0,C26-E26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="B27" s="12" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C27" s="12">
+        <f>1000*A27*'1 Inputs'!$B$26</f>
+        <v/>
+      </c>
+      <c r="D27" s="12">
+        <f>MAX(0,'1 Inputs'!$B$5-B27)</f>
+        <v/>
+      </c>
+      <c r="E27" s="12">
+        <f>MIN(C27,D27)</f>
+        <v/>
+      </c>
+      <c r="F27" s="12">
+        <f>MAX(0,C27-E27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="B28" s="12" t="n">
+        <v>1400</v>
+      </c>
+      <c r="C28" s="12">
+        <f>1000*A28*'1 Inputs'!$B$26</f>
+        <v/>
+      </c>
+      <c r="D28" s="12">
+        <f>MAX(0,'1 Inputs'!$B$5-B28)</f>
+        <v/>
+      </c>
+      <c r="E28" s="12">
+        <f>MIN(C28,D28)</f>
+        <v/>
+      </c>
+      <c r="F28" s="12">
+        <f>MAX(0,C28-E28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="16" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="B29" s="12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C29" s="12">
+        <f>1000*A29*'1 Inputs'!$B$26</f>
+        <v/>
+      </c>
+      <c r="D29" s="12">
+        <f>MAX(0,'1 Inputs'!$B$5-B29)</f>
+        <v/>
+      </c>
+      <c r="E29" s="12">
+        <f>MIN(C29,D29)</f>
+        <v/>
+      </c>
+      <c r="F29" s="12">
+        <f>MAX(0,C29-E29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="B30" s="12" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C30" s="12">
+        <f>1000*A30*'1 Inputs'!$B$26</f>
+        <v/>
+      </c>
+      <c r="D30" s="12">
+        <f>MAX(0,'1 Inputs'!$B$5-B30)</f>
+        <v/>
+      </c>
+      <c r="E30" s="12">
+        <f>MIN(C30,D30)</f>
+        <v/>
+      </c>
+      <c r="F30" s="12">
+        <f>MAX(0,C30-E30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="B31" s="12" t="n">
+        <v>1400</v>
+      </c>
+      <c r="C31" s="12">
+        <f>1000*A31*'1 Inputs'!$B$26</f>
+        <v/>
+      </c>
+      <c r="D31" s="12">
+        <f>MAX(0,'1 Inputs'!$B$5-B31)</f>
+        <v/>
+      </c>
+      <c r="E31" s="12">
+        <f>MIN(C31,D31)</f>
+        <v/>
+      </c>
+      <c r="F31" s="12">
+        <f>MAX(0,C31-E31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>PG UNIT ECONOMICS — EXISTING MODEL AOV REFERENCES, NOT A FORECAST</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>AOV reference</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>AOV</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Common-drop share</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Last mile</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Contribution/order</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>Minutes current midpoint</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="n">
+        <v>450</v>
+      </c>
+      <c r="C36" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="13">
+        <f>(1-C36)*'1 Inputs'!$B$27+C36*'1 Inputs'!$B$28</f>
+        <v/>
+      </c>
+      <c r="E36" s="13">
+        <f>'1 Inputs'!$B$8*B36-D36-'1 Inputs'!$B$10-'1 Inputs'!$B$11-'1 Inputs'!$B$12</f>
+        <v/>
+      </c>
+      <c r="F36" s="8">
+        <f>IF(E36&gt;0,"positive before fixed cost","does not cover variable cost")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>Minutes current midpoint</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="n">
+        <v>450</v>
+      </c>
+      <c r="C37" s="16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D37" s="13">
+        <f>(1-C37)*'1 Inputs'!$B$27+C37*'1 Inputs'!$B$28</f>
+        <v/>
+      </c>
+      <c r="E37" s="13">
+        <f>'1 Inputs'!$B$8*B37-D37-'1 Inputs'!$B$10-'1 Inputs'!$B$11-'1 Inputs'!$B$12</f>
+        <v/>
+      </c>
+      <c r="F37" s="8">
+        <f>IF(E37&gt;0,"positive before fixed cost","does not cover variable cost")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>Minutes current midpoint</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="n">
+        <v>450</v>
+      </c>
+      <c r="C38" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="13">
+        <f>(1-C38)*'1 Inputs'!$B$27+C38*'1 Inputs'!$B$28</f>
+        <v/>
+      </c>
+      <c r="E38" s="13">
+        <f>'1 Inputs'!$B$8*B38-D38-'1 Inputs'!$B$10-'1 Inputs'!$B$11-'1 Inputs'!$B$12</f>
+        <v/>
+      </c>
+      <c r="F38" s="8">
+        <f>IF(E38&gt;0,"positive before fixed cost","does not cover variable cost")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>Campus spine breakeven</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="n">
+        <v>573.0960959462569</v>
+      </c>
+      <c r="C39" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" s="13">
+        <f>(1-C39)*'1 Inputs'!$B$27+C39*'1 Inputs'!$B$28</f>
+        <v/>
+      </c>
+      <c r="E39" s="13">
+        <f>'1 Inputs'!$B$8*B39-D39-'1 Inputs'!$B$10-'1 Inputs'!$B$11-'1 Inputs'!$B$12</f>
+        <v/>
+      </c>
+      <c r="F39" s="8">
+        <f>IF(E39&gt;0,"positive before fixed cost","does not cover variable cost")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>Campus spine breakeven</t>
+        </is>
+      </c>
+      <c r="B40" s="13" t="n">
+        <v>573.0960959462569</v>
+      </c>
+      <c r="C40" s="16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D40" s="13">
+        <f>(1-C40)*'1 Inputs'!$B$27+C40*'1 Inputs'!$B$28</f>
+        <v/>
+      </c>
+      <c r="E40" s="13">
+        <f>'1 Inputs'!$B$8*B40-D40-'1 Inputs'!$B$10-'1 Inputs'!$B$11-'1 Inputs'!$B$12</f>
+        <v/>
+      </c>
+      <c r="F40" s="8">
+        <f>IF(E40&gt;0,"positive before fixed cost","does not cover variable cost")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>Campus spine breakeven</t>
+        </is>
+      </c>
+      <c r="B41" s="13" t="n">
+        <v>573.0960959462569</v>
+      </c>
+      <c r="C41" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="13">
+        <f>(1-C41)*'1 Inputs'!$B$27+C41*'1 Inputs'!$B$28</f>
+        <v/>
+      </c>
+      <c r="E41" s="13">
+        <f>'1 Inputs'!$B$8*B41-D41-'1 Inputs'!$B$10-'1 Inputs'!$B$11-'1 Inputs'!$B$12</f>
+        <v/>
+      </c>
+      <c r="F41" s="8">
+        <f>IF(E41&gt;0,"positive before fixed cost","does not cover variable cost")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>30% non-grocery basket</t>
+        </is>
+      </c>
+      <c r="B42" s="13" t="n">
+        <v>729.383462929356</v>
+      </c>
+      <c r="C42" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" s="13">
+        <f>(1-C42)*'1 Inputs'!$B$27+C42*'1 Inputs'!$B$28</f>
+        <v/>
+      </c>
+      <c r="E42" s="13">
+        <f>'1 Inputs'!$B$8*B42-D42-'1 Inputs'!$B$10-'1 Inputs'!$B$11-'1 Inputs'!$B$12</f>
+        <v/>
+      </c>
+      <c r="F42" s="8">
+        <f>IF(E42&gt;0,"positive before fixed cost","does not cover variable cost")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>30% non-grocery basket</t>
+        </is>
+      </c>
+      <c r="B43" s="13" t="n">
+        <v>729.383462929356</v>
+      </c>
+      <c r="C43" s="16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D43" s="13">
+        <f>(1-C43)*'1 Inputs'!$B$27+C43*'1 Inputs'!$B$28</f>
+        <v/>
+      </c>
+      <c r="E43" s="13">
+        <f>'1 Inputs'!$B$8*B43-D43-'1 Inputs'!$B$10-'1 Inputs'!$B$11-'1 Inputs'!$B$12</f>
+        <v/>
+      </c>
+      <c r="F43" s="8">
+        <f>IF(E43&gt;0,"positive before fixed cost","does not cover variable cost")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>30% non-grocery basket</t>
+        </is>
+      </c>
+      <c r="B44" s="13" t="n">
+        <v>729.383462929356</v>
+      </c>
+      <c r="C44" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="13">
+        <f>(1-C44)*'1 Inputs'!$B$27+C44*'1 Inputs'!$B$28</f>
+        <v/>
+      </c>
+      <c r="E44" s="13">
+        <f>'1 Inputs'!$B$8*B44-D44-'1 Inputs'!$B$10-'1 Inputs'!$B$11-'1 Inputs'!$B$12</f>
+        <v/>
+      </c>
+      <c r="F44" s="8">
+        <f>IF(E44&gt;0,"positive before fixed cost","does not cover variable cost")</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -708,7 +1580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1106,6 +1978,356 @@
       <c r="E18" s="6" t="inlineStr">
         <is>
           <t>must outlive its own payback</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>PG demand evidence gate</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>TRUE/FALSE</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>opens only after site evidence is approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>PG verified occupied student beds</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>beds</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>occupied STUDENT beds inside the served radius</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>PG active-user penetration</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>pilot-observed active users / occupied student beds</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>PG gross AOV</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Rs/order</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>pilot-observed; zero means not evidenced</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>PG common-drop share</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>share served at reception, warden desk or locker</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>PG break retention</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>% of term</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>PG demand persisting through the academic break</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Hostel term volume in PG scenario</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>1400</v>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>orders/day</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>capacity already consumed by the hostel base</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>PG orders per active user per day</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>orders/day</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>Blinkit 3.6/month / 30; no captive-campus uplift</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>PG doorstep last mile</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="n">
+        <v>26.87389770723104</v>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Rs/order</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>cost_stack Type B urban PG geometry</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>PG common-drop last mile</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="n">
+        <v>23.95282186948853</v>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Rs/order</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>cost_stack Type B common-drop geometry</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>NOV / GOV</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="n">
+        <v>0.791</v>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>Blinkit FY26E</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Term days</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="n">
+        <v>258.5416666666667</v>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>days/year</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>365 x active academic months / 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Break days</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="n">
+        <v>106.4583333333333</v>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>days/year</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>365 - term days</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Hostel comparison AOV</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="n">
+        <v>729.383462929356</v>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Rs/order</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>basket at the 30% non-grocery floor</t>
         </is>
       </c>
     </row>
@@ -1205,222 +2427,222 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Peak (late evening, exam windows)</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n">
+      <c r="B5" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="8" t="n">
         <v>0.6274509803921569</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="E5" s="8" t="n">
         <v>103.7</v>
       </c>
-      <c r="F5" s="7" t="n">
+      <c r="F5" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="G5" s="7" t="n">
+      <c r="G5" s="8" t="n">
         <v>5.12</v>
       </c>
-      <c r="H5" s="7" t="n">
+      <c r="H5" s="8" t="n">
         <v>3.36</v>
       </c>
-      <c r="I5" s="7" t="n">
+      <c r="I5" s="8" t="n">
         <v>8.48</v>
       </c>
-      <c r="J5" s="7" t="n">
+      <c r="J5" s="8" t="n">
         <v>27.1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="8" t="n">
         <v>0.3137254901960784</v>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E6" s="8" t="n">
         <v>25.9</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="F6" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G6" s="7" t="n">
+      <c r="G6" s="8" t="n">
         <v>25.59</v>
       </c>
-      <c r="H6" s="7" t="n">
+      <c r="H6" s="8" t="n">
         <v>3.36</v>
       </c>
-      <c r="I6" s="7" t="n">
+      <c r="I6" s="8" t="n">
         <v>28.95</v>
       </c>
-      <c r="J6" s="7" t="n">
+      <c r="J6" s="8" t="n">
         <v>21.6</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Trough (early morning, class hrs)</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="8" t="n">
         <v>0.25</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="8" t="n">
         <v>0.05882352941176471</v>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="E7" s="8" t="n">
         <v>6.5</v>
       </c>
-      <c r="F7" s="7" t="n">
+      <c r="F7" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="7" t="n">
+      <c r="G7" s="8" t="n">
         <v>51.18</v>
       </c>
-      <c r="H7" s="7" t="n">
+      <c r="H7" s="8" t="n">
         <v>3.36</v>
       </c>
-      <c r="I7" s="7" t="n">
+      <c r="I7" s="8" t="n">
         <v>54.54</v>
       </c>
-      <c r="J7" s="7" t="n">
+      <c r="J7" s="8" t="n">
         <v>25.7</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>VOLUME-WEIGHTED LAST MILE</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n"/>
-      <c r="C9" s="8" t="n"/>
-      <c r="D9" s="8" t="n"/>
-      <c r="E9" s="8" t="n"/>
-      <c r="F9" s="8" t="n"/>
-      <c r="G9" s="8">
+      <c r="B9" s="9" t="n"/>
+      <c r="C9" s="9" t="n"/>
+      <c r="D9" s="9" t="n"/>
+      <c r="E9" s="9" t="n"/>
+      <c r="F9" s="9" t="n"/>
+      <c r="G9" s="9">
         <f>SUMPRODUCT(D5:D7,G5:G7)</f>
         <v/>
       </c>
-      <c r="H9" s="8">
+      <c r="H9" s="9">
         <f>H5</f>
         <v/>
       </c>
-      <c r="I9" s="8">
+      <c r="I9" s="9">
         <f>G9+H9</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Standard 2–3 km residential zone</t>
         </is>
       </c>
-      <c r="B10" s="9" t="n"/>
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="9" t="n"/>
-      <c r="E10" s="9" t="n"/>
-      <c r="F10" s="9" t="n"/>
-      <c r="G10" s="9" t="n"/>
-      <c r="H10" s="9" t="n"/>
-      <c r="I10" s="9" t="n">
+      <c r="B10" s="10" t="n"/>
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="10" t="n"/>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="n"/>
+      <c r="G10" s="10" t="n"/>
+      <c r="H10" s="10" t="n"/>
+      <c r="I10" s="10" t="n">
         <v>42</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Saving vs a standard zone</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n"/>
-      <c r="C11" s="8" t="n"/>
-      <c r="D11" s="8" t="n"/>
-      <c r="E11" s="8" t="n"/>
-      <c r="F11" s="8" t="n"/>
-      <c r="G11" s="8" t="n"/>
-      <c r="H11" s="8" t="n"/>
-      <c r="I11" s="8">
+      <c r="B11" s="9" t="n"/>
+      <c r="C11" s="9" t="n"/>
+      <c r="D11" s="9" t="n"/>
+      <c r="E11" s="9" t="n"/>
+      <c r="F11" s="9" t="n"/>
+      <c r="G11" s="9" t="n"/>
+      <c r="H11" s="9" t="n"/>
+      <c r="I11" s="9">
         <f>1-I9/I10</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>ROSTER — base case is PER GATE</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n"/>
-      <c r="C14" s="8" t="n"/>
-      <c r="D14" s="8" t="n"/>
-      <c r="E14" s="8" t="n"/>
+      <c r="B14" s="9" t="n"/>
+      <c r="C14" s="9" t="n"/>
+      <c r="D14" s="9" t="n"/>
+      <c r="E14" s="9" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>per gate (467/day)</t>
         </is>
       </c>
-      <c r="B15" s="9" t="n">
+      <c r="B15" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>runners</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>alpha 87%</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>Rs3.36/order</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>pooled across 3 gates (UPSIDE, not the plan)</t>
         </is>
       </c>
-      <c r="B16" s="9" t="n">
+      <c r="B16" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>runners</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D16" s="10" t="inlineStr">
         <is>
           <t>alpha 100%</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E16" s="10" t="inlineStr">
         <is>
           <t>Rs2.88/order — Rs0.48 better, conditional on cross-gate movement</t>
         </is>
@@ -1486,180 +2708,180 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Variable cost per order</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n">
+      <c r="B5" s="8" t="n">
         <v>80.92</v>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Rs</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>last mile + store ops + packaging + residual</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Active days per year</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="8" t="n">
         <v>258.5</v>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>days</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>365 x 8.5/12</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Annual orders, term-only</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="8" t="n">
         <v>361958</v>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>orders</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>returns basis</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Breakeven AOV — 365-day returns basis</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="8" t="n">
         <v>571</v>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>Rs</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>ROCE = 0</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Breakeven AOV — 30-day deck spine</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="8" t="n">
         <v>573</v>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>Rs</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>the deck headline</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Day-count gap between the two</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n">
+      <c r="B10" s="8" t="n">
         <v>2.14</v>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Rs</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>asserted, not smoothed</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>AOV at the 40% external benchmark</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n">
+      <c r="B11" s="8" t="n">
         <v>755</v>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Rs</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>Eternal's disclosed return, not Flipkart's</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>Premium over breakeven</t>
         </is>
       </c>
-      <c r="B12" s="7" t="n">
+      <c r="B12" s="8" t="n">
         <v>184</v>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>Rs</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>what the basket lever must buy</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Non-grocery share the benchmark implies</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n">
+      <c r="B13" s="8" t="n">
         <v>32.3</v>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>% of GOV</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>inside the 30-40% range Swiggy discloses</t>
         </is>
@@ -1727,136 +2949,136 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Capex, band midpoint</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n">
+      <c r="B5" s="8" t="n">
         <v>235</v>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Rs lakh</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr"/>
+      <c r="D5" s="8" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Working capital</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="8" t="n">
         <v>88.90000000000001</v>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>Rs lakh</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>14 NWC days on NOV</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Capital employed</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="8" t="n">
         <v>323.9</v>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Rs lakh</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>capex + working capital</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>DuPont margin leg</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="8" t="n">
         <v>4.74</v>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>at the benchmark AOV</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>DuPont turnover leg</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="8" t="n">
         <v>8.44</v>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>the node's own turnover on CE</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Like-for-like asset turn</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n">
+      <c r="B10" s="8" t="n">
         <v>6.93</v>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>common AOV Rs450, isolates density x calendar</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>IRR at the benchmark AOV</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n">
+      <c r="B11" s="8" t="n">
         <v>34.4</v>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>5-year life, 3-month ramp</t>
         </is>
@@ -1895,92 +3117,92 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>Underwritten  (AOV at breakeven)</t>
         </is>
       </c>
-      <c r="B14" s="9" t="n">
+      <c r="B14" s="10" t="n">
         <v>571</v>
       </c>
-      <c r="C14" s="9" t="n">
+      <c r="C14" s="10" t="n">
         <v>-0</v>
       </c>
-      <c r="D14" s="9" t="n">
+      <c r="D14" s="10" t="n">
         <v>6.38</v>
       </c>
-      <c r="E14" s="9" t="n">
+      <c r="E14" s="10" t="n">
         <v>-0</v>
       </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="F14" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>Basket at 30% non-grocery</t>
         </is>
       </c>
-      <c r="B15" s="9" t="n">
+      <c r="B15" s="10" t="n">
         <v>729</v>
       </c>
-      <c r="C15" s="9" t="n">
+      <c r="C15" s="10" t="n">
         <v>4.22</v>
       </c>
-      <c r="D15" s="9" t="n">
+      <c r="D15" s="10" t="n">
         <v>8.15</v>
       </c>
-      <c r="E15" s="9" t="n">
+      <c r="E15" s="10" t="n">
         <v>34.4</v>
       </c>
-      <c r="F15" s="9" t="n">
+      <c r="F15" s="10" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>Basket at 40% non-grocery</t>
         </is>
       </c>
-      <c r="B16" s="9" t="n">
+      <c r="B16" s="10" t="n">
         <v>842</v>
       </c>
-      <c r="C16" s="9" t="n">
+      <c r="C16" s="10" t="n">
         <v>6.25</v>
       </c>
-      <c r="D16" s="9" t="n">
+      <c r="D16" s="10" t="n">
         <v>9.41</v>
       </c>
-      <c r="E16" s="9" t="n">
+      <c r="E16" s="10" t="n">
         <v>58.8</v>
       </c>
-      <c r="F16" s="9" t="n">
+      <c r="F16" s="10" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>Basket at 30%, volume -30%</t>
         </is>
       </c>
-      <c r="B17" s="9" t="n">
+      <c r="B17" s="10" t="n">
         <v>729</v>
       </c>
-      <c r="C17" s="9" t="n">
+      <c r="C17" s="10" t="n">
         <v>2.46</v>
       </c>
-      <c r="D17" s="9" t="n">
+      <c r="D17" s="10" t="n">
         <v>5.71</v>
       </c>
-      <c r="E17" s="9" t="n">
+      <c r="E17" s="10" t="n">
         <v>14</v>
       </c>
-      <c r="F17" s="9" t="n">
+      <c r="F17" s="10" t="n">
         <v>62</v>
       </c>
     </row>
@@ -2045,99 +3267,99 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>credit intact</t>
         </is>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>suppliers resume terms; the rebuild is payables-funded</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>30-day reset</t>
         </is>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="10" t="n">
         <v>37.8</v>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>partially self-funded while terms re-establish</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>full reset (ADOPTED)</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="8" t="n">
         <v>75.5</v>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>the whole 60-day cycle self-funded — the downside</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Working-capital constructs</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n"/>
-      <c r="C9" s="8" t="n"/>
+      <c r="B9" s="9" t="n"/>
+      <c r="C9" s="9" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>NWC days x NOV (14d)</t>
         </is>
       </c>
-      <c r="B10" s="9" t="n">
+      <c r="B10" s="10" t="n">
         <v>88.90000000000001</v>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>ADOPTED</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>12-day steady state</t>
         </is>
       </c>
-      <c r="B11" s="9" t="n">
+      <c r="B11" s="10" t="n">
         <v>76.2</v>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>sensitivity</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>COGS x 18 days</t>
         </is>
       </c>
-      <c r="B12" s="9" t="n">
+      <c r="B12" s="10" t="n">
         <v>116.4</v>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>REJECTED — double-counts the netting</t>
         </is>
@@ -2197,60 +3419,60 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Volume -30%</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n">
+      <c r="B5" s="8" t="n">
         <v>640</v>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>thinner fixed-base absorption</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Shrinkage, upper bound</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="8" t="n">
         <v>615</v>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>1.8% of NOV</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Gig social-security levy</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="8" t="n">
         <v>588</v>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>201st Parliamentary report</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Calendar fragmentation</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="8" t="n">
         <v>582</v>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>shape of the break, not its length</t>
         </is>
@@ -2317,101 +3539,101 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Institutions in the register</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n">
+      <c r="B5" s="8" t="n">
         <v>72352</v>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>AISHE, as on 28-8-2026</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Colleges only</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="8" t="n">
         <v>54014</v>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>colleges</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Urban colleges</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="8" t="n">
         <v>21000</v>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>urban flag</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Districts passing four criteria</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="8" t="n">
         <v>111</v>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>of 765 (State, District) pairs</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Uncontested</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>the screen's own floor: 6-7 urban colleges</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Contested</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n">
+      <c r="B10" s="8" t="n">
         <v>22</v>
       </c>
-      <c r="C10" s="7" t="inlineStr"/>
+      <c r="C10" s="8" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Stacked</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n">
+      <c r="B11" s="8" t="n">
         <v>80</v>
       </c>
-      <c r="C11" s="7" t="inlineStr"/>
+      <c r="C11" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2461,108 +3683,108 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>params.py</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>a contested policy constant defined more than once</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>verify_artifacts.py</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>a stale figure in the workbook, notebooks or asset manifest</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>recon(a, b)</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>two modules computing the same quantity under different policies</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>phrase bans</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>wording the deck must not contain, including attribution</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>superseded-value bans</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>a pre-correction figure surviving in any panel</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>duplicate-registration guard</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>a check registered twice, inflating the count</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>stale-basis scan</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>a superseded value used as a literal cost basis, defaults included</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>document scan</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>a superseded figure in HANDOFF, spec, build prompt or README</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>release.py</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>build - verify - capture - stamp - re-verify the exact stamped file</t>
         </is>

</xml_diff>

<commit_message>
Add evidence-gated demand-state assortment model
</commit_message>
<xml_diff>
--- a/Campus_Store_Model.xlsx
+++ b/Campus_Store_Model.xlsx
@@ -17,6 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7 District Screen" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8 Verification" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9 PG Adjacency" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Assortment" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -117,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -139,6 +140,7 @@
     <xf numFmtId="3" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1574,13 +1576,744 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Assortment — demand-state local range, wide network promise</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>The optimiser changes what is held locally, not what the Minutes network can offer. All 16,500 network SKUs remain available through SDFC backfill. Financial savings remain zero until the gold pilot inputs on 1 Inputs are evidenced and explicitly promoted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>FINANCIAL PROMOTION GATE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Decision reading</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>Evidence status</t>
+        </is>
+      </c>
+      <c r="B6" s="11">
+        <f>IF(AND('1 Inputs'!$B$33=TRUE,OR('1 Inputs'!$B$34&gt;0,'1 Inputs'!$B$35&gt;0,'1 Inputs'!$B$36&gt;0)),"OPEN","CLOSED")</f>
+        <v/>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>CLOSED means no assortment saving enters the published solver</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Incremental monthly opex saving</t>
+        </is>
+      </c>
+      <c r="B7" s="14">
+        <f>IF(B6="OPEN",'1 Inputs'!$B$34+'1 Inputs'!$B$35,0)</f>
+        <v/>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>excludes the cold-power saving already in break_mode.cfg_cold</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>One-time NWC release</t>
+        </is>
+      </c>
+      <c r="B8" s="14">
+        <f>IF(B6="OPEN",'1 Inputs'!$B$36,0)</f>
+        <v/>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>cash timing only; not EBIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Promoted to solver</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>requires a separate reviewed promotion decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>OPTIMISED LOCAL SKU ALLOCATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Temperature</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Trough</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Peak</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Break</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Ambient staples</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>ambient</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="n">
+        <v>2757</v>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>2965</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>2734</v>
+      </c>
+      <c r="F14" s="14" t="n">
+        <v>2650</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <v>2268</v>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>A — policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Chilled / ready-to-eat</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>chilled</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="n">
+        <v>668</v>
+      </c>
+      <c r="D15" s="14" t="n">
+        <v>923</v>
+      </c>
+      <c r="E15" s="14" t="n">
+        <v>1067</v>
+      </c>
+      <c r="F15" s="14" t="n">
+        <v>934</v>
+      </c>
+      <c r="G15" s="14" t="n">
+        <v>250</v>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>A — policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Frozen snacks</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>frozen</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="n">
+        <v>498</v>
+      </c>
+      <c r="D16" s="14" t="n">
+        <v>651</v>
+      </c>
+      <c r="E16" s="14" t="n">
+        <v>799</v>
+      </c>
+      <c r="F16" s="14" t="n">
+        <v>651</v>
+      </c>
+      <c r="G16" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>A — policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Fresh / perishables</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>chilled</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="n">
+        <v>634</v>
+      </c>
+      <c r="D17" s="14" t="n">
+        <v>726</v>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>634</v>
+      </c>
+      <c r="F17" s="14" t="n">
+        <v>615</v>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>150</v>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>A — policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Snacks / caffeine</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>ambient</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="n">
+        <v>1150</v>
+      </c>
+      <c r="D18" s="14" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E18" s="14" t="n">
+        <v>1600</v>
+      </c>
+      <c r="F18" s="14" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>732</v>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>A — policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>BPC / stationery / print</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>ambient</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="n">
+        <v>801</v>
+      </c>
+      <c r="D19" s="14" t="n">
+        <v>801</v>
+      </c>
+      <c r="E19" s="14" t="n">
+        <v>801</v>
+      </c>
+      <c r="F19" s="14" t="n">
+        <v>1200</v>
+      </c>
+      <c r="G19" s="14" t="n">
+        <v>450</v>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>A — policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Local long tail</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>ambient</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="n">
+        <v>492</v>
+      </c>
+      <c r="D20" s="14" t="n">
+        <v>634</v>
+      </c>
+      <c r="E20" s="14" t="n">
+        <v>365</v>
+      </c>
+      <c r="F20" s="14" t="n">
+        <v>350</v>
+      </c>
+      <c r="G20" s="14" t="n">
+        <v>250</v>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>A — policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>LOCAL SKUs</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C21" s="9">
+        <f>SUM(C14:C20)</f>
+        <v/>
+      </c>
+      <c r="D21" s="9">
+        <f>SUM(D14:D20)</f>
+        <v/>
+      </c>
+      <c r="E21" s="9">
+        <f>SUM(E14:E20)</f>
+        <v/>
+      </c>
+      <c r="F21" s="9">
+        <f>SUM(F14:F20)</f>
+        <v/>
+      </c>
+      <c r="G21" s="9">
+        <f>SUM(G14:G20)</f>
+        <v/>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>computed</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>SDFC tail</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C22" s="5">
+        <f>16500-C21</f>
+        <v/>
+      </c>
+      <c r="D22" s="5">
+        <f>16500-D21</f>
+        <v/>
+      </c>
+      <c r="E22" s="5">
+        <f>16500-E21</f>
+        <v/>
+      </c>
+      <c r="F22" s="5">
+        <f>16500-F21</f>
+        <v/>
+      </c>
+      <c r="G22" s="5">
+        <f>16500-G21</f>
+        <v/>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>computed</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>NETWORK assortment</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C23" s="17">
+        <f>C21+C22</f>
+        <v/>
+      </c>
+      <c r="D23" s="17">
+        <f>D21+D22</f>
+        <v/>
+      </c>
+      <c r="E23" s="17">
+        <f>E21+E22</f>
+        <v/>
+      </c>
+      <c r="F23" s="17">
+        <f>F21+F22</f>
+        <v/>
+      </c>
+      <c r="G23" s="17">
+        <f>G21+G22</f>
+        <v/>
+      </c>
+      <c r="H23" s="17" t="inlineStr">
+        <is>
+          <t>must remain wide</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Cold SKUs</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C24" s="5">
+        <f>SUM(C15:C17)</f>
+        <v/>
+      </c>
+      <c r="D24" s="5">
+        <f>SUM(D15:D17)</f>
+        <v/>
+      </c>
+      <c r="E24" s="5">
+        <f>SUM(E15:E17)</f>
+        <v/>
+      </c>
+      <c r="F24" s="5">
+        <f>SUM(F15:F17)</f>
+        <v/>
+      </c>
+      <c r="G24" s="5">
+        <f>SUM(G15:G17)</f>
+        <v/>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>chilled + frozen</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Local cap</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>7000</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>8000</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>8000</v>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>4200</v>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>hard constraint</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Cold cap</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>1800</v>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>2300</v>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>700</v>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>hard constraint</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Guardrail</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C27" s="11">
+        <f>IF(AND(C21&lt;=C25,C24&lt;=C26,C23=16500),"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="D27" s="11">
+        <f>IF(AND(D21&lt;=D25,D24&lt;=D26,D23=16500),"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="E27" s="11">
+        <f>IF(AND(E21&lt;=E25,E24&lt;=E26,E23=16500),"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="F27" s="11">
+        <f>IF(AND(F21&lt;=F25,F24&lt;=F26,F23=16500),"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="G27" s="11">
+        <f>IF(AND(G21&lt;=G25,G24&lt;=G26,G23=16500),"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="H27" s="11" t="inlineStr">
+        <is>
+          <t>all three must hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>PILOT DATA REQUIRED BEFORE FINANCIAL PROMOTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Why it matters</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>Category velocity by demand state</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>replaces A-tier priorities with observed demand</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>Waste and markdown by category</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>prices only genuinely avoided loss</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>Shelf life, case pack and replenishment lead</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>sets safe inventory floors</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>Cold-zone kWh by operating mode</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>reconciles with, rather than duplicates, cfg_cold</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>Stockout and fill-rate guardrails</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>prevents cost savings from weakening the promise</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:H2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2328,6 +3061,106 @@
       <c r="E32" s="6" t="inlineStr">
         <is>
           <t>basket at the 30% non-grocery floor</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Assortment financial evidence gate</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>TRUE/FALSE</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>opens only after pilot category evidence is approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>Assortment waste + markdown saving</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Rs/break month</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>pilot-observed; zero means not evidenced</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>Assortment handling saving</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Rs/break month</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>pilot-observed; excludes labour already flexed elsewhere</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>Assortment NWC release</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Rs one-time</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>pilot-observed cash release; not EBIT</t>
         </is>
       </c>
     </row>

</xml_diff>